<commit_message>
Decouple backend API and static frontend components
</commit_message>
<xml_diff>
--- a/uploads/IT_4.xlsx
+++ b/uploads/IT_4.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\moham\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/62d0963de6c5dd7b/Desktop/lc_tracker/uploads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{625D7B0E-77DE-4AEF-AAD7-874AB3CA4124}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:1_{625D7B0E-77DE-4AEF-AAD7-874AB3CA4124}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9346685E-B237-4687-AEAD-4947FEE8A5ED}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="72">
   <si>
     <t xml:space="preserve">KALYANI J </t>
   </si>
@@ -187,9 +187,6 @@
     <t xml:space="preserve">Daksatha M </t>
   </si>
   <si>
-    <t xml:space="preserve">Daksatha </t>
-  </si>
-  <si>
     <t xml:space="preserve">Ashokkumar T </t>
   </si>
   <si>
@@ -224,6 +221,21 @@
   </si>
   <si>
     <t>Name</t>
+  </si>
+  <si>
+    <t>Bharath Raj T</t>
+  </si>
+  <si>
+    <t>BHARATHRAJ_2005</t>
+  </si>
+  <si>
+    <t>Mohamed Halid P</t>
+  </si>
+  <si>
+    <t>mohamedhalid</t>
+  </si>
+  <si>
+    <t>Daksatha25</t>
   </si>
 </sst>
 </file>
@@ -330,7 +342,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Form_Responses" displayName="Form_Responses" ref="A1:C35">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Form_Responses" displayName="Form_Responses" ref="A1:C37">
   <tableColumns count="3">
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Name"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Register Number"/>
@@ -541,7 +553,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="10" width="18.88671875" customWidth="1"/>
@@ -549,13 +561,13 @@
   <sheetData>
     <row r="1" spans="1:3" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -874,62 +886,84 @@
         <v>721023205011</v>
       </c>
       <c r="C30" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B31">
         <v>721023205008</v>
       </c>
       <c r="C31" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B32">
         <v>721023205003</v>
       </c>
       <c r="C32" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B33">
         <v>721023205026</v>
       </c>
       <c r="C33" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B34">
         <v>721023205016</v>
       </c>
       <c r="C34" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B35">
         <v>721023205057</v>
       </c>
       <c r="C35" t="s">
-        <v>64</v>
+        <v>63</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>67</v>
+      </c>
+      <c r="B36">
+        <v>721023205009</v>
+      </c>
+      <c r="C36" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>69</v>
+      </c>
+      <c r="B37">
+        <v>721023205039</v>
+      </c>
+      <c r="C37" t="s">
+        <v>70</v>
       </c>
     </row>
   </sheetData>

</xml_diff>